<commit_message>
WIP: source workbooks singular + outline groups + MC total section; extractor invariant 6
- All four workbooks: "Member's Capital" singular everywhere (8 title/label
  cells); Excel outline groups on the sorted Steps sheets (IS 2/4, CF 2/3)
  so rendered working sheets collapse; Members-Capital-Steps final mirrors
  Rick's total section (2,460 / +2,040 / 4,500); Balance Sheet converted to
  hard values (Rick), with correct MC-section figures.
- extract-statement-steps.py: invariant 6 — every Balance Sheet line must
  equal its ledger's dated ruled balances (17 comparisons), replacing the
  live-formula drift protection.
- Regenerated data: all 6 invariants green; zero plural strings.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bike-Repair-Source-Workbooks/Bike-Repair-End.xlsx
+++ b/Bike-Repair-Source-Workbooks/Bike-Repair-End.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ra1/Courses-Local/Instructional_Redesign_v2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ra1/Courses-Local/Instructional_Redesign_v2/Bike-Repair-Source-Workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6957ADFD-630D-3941-8745-87D8653D9B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_8AACC1A09D727DA7503BA1B526C6193B2695CC45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15540" yWindow="2240" windowWidth="26120" windowHeight="27720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15540" yWindow="2240" windowWidth="26120" windowHeight="27720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assets" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,46 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="188">
+  <si>
+    <t>[Your Name]'s Bike Repair, LLC.</t>
+  </si>
+  <si>
+    <t>Statement of Member's Capital</t>
+  </si>
+  <si>
+    <t>For the period June 1 – August 31, 2026</t>
+  </si>
+  <si>
+    <t>CONTRIBUTED</t>
+  </si>
+  <si>
+    <t>Balance, June 1, 2026</t>
+  </si>
+  <si>
+    <t>Balance, August 31, 2026</t>
+  </si>
+  <si>
+    <t>GENERATED</t>
+  </si>
+  <si>
+    <t>Net income (from the Income Statement)</t>
+  </si>
+  <si>
+    <t>WITHDRAWN</t>
+  </si>
+  <si>
+    <t>Owner's draw</t>
+  </si>
+  <si>
+    <t>Total Member's Capital, June 1, 2026</t>
+  </si>
+  <si>
+    <t>Change in total Member's Capital, June 1 to August 31, 2026</t>
+  </si>
+  <si>
+    <t>Total Member's Capital, August 31, 2026</t>
+  </si>
   <si>
     <t>Assets</t>
   </si>
@@ -65,9 +104,6 @@
     <t>Deposited to open the LLC bank account</t>
   </si>
   <si>
-    <t>Balance, June 1, 2026</t>
-  </si>
-  <si>
     <t>Repair collected — Dana R.</t>
   </si>
   <si>
@@ -152,9 +188,6 @@
     <t>Money taken out for personal use</t>
   </si>
   <si>
-    <t>Balance, August 31, 2026</t>
-  </si>
-  <si>
     <t>Accounts Receivable</t>
   </si>
   <si>
@@ -398,10 +431,7 @@
     <t>Built and delivered Smith's frame — no longer owed</t>
   </si>
   <si>
-    <t>Reasons — Members' Capital</t>
-  </si>
-  <si>
-    <t>CONTRIBUTED</t>
+    <t>Reasons — Member's Capital</t>
   </si>
   <si>
     <t>Cash — covered from your personal funds (May)</t>
@@ -416,9 +446,6 @@
     <t>Cash — deposited to open the LLC bank account (June 1)</t>
   </si>
   <si>
-    <t>GENERATED</t>
-  </si>
-  <si>
     <t>Repair collected — Brake job + Tune-up + Tire mounting ×2 @ $70</t>
   </si>
   <si>
@@ -470,15 +497,9 @@
     <t>Depreciation — laptop, Summer 2026</t>
   </si>
   <si>
-    <t>WITHDRAWN</t>
-  </si>
-  <si>
     <t>Owner's draw — money taken out for personal use</t>
   </si>
   <si>
-    <t>[Your Name]'s Bike Repair, LLC.</t>
-  </si>
-  <si>
     <t>Balance Sheets</t>
   </si>
   <si>
@@ -494,7 +515,7 @@
     <t>Total Liabilities</t>
   </si>
   <si>
-    <t>Members' Capital</t>
+    <t>Member's Capital</t>
   </si>
   <si>
     <t>Contributed</t>
@@ -506,15 +527,12 @@
     <t>Withdrawn</t>
   </si>
   <si>
-    <t>Total Members' Capital</t>
+    <t>Total Member's Capital</t>
   </si>
   <si>
     <t>Income Statement</t>
   </si>
   <si>
-    <t>For the period June 1 – August 31, 2026</t>
-  </si>
-  <si>
     <t>Revenue</t>
   </si>
   <si>
@@ -540,15 +558,6 @@
   </si>
   <si>
     <t>Net income</t>
-  </si>
-  <si>
-    <t>Statement of Members' Capital</t>
-  </si>
-  <si>
-    <t>Net income (from the Income Statement)</t>
-  </si>
-  <si>
-    <t>Owner's draw</t>
   </si>
   <si>
     <t>Cash Flow Statement</t>
@@ -695,7 +704,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -723,11 +732,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -770,6 +790,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1086,19 +1107,19 @@
   <sheetData>
     <row r="1" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D3" s="4">
         <v>-1300</v>
@@ -1106,7 +1127,7 @@
     </row>
     <row r="4" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D4" s="4">
         <v>-200</v>
@@ -1114,7 +1135,7 @@
     </row>
     <row r="5" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D5" s="4">
         <v>340</v>
@@ -1122,7 +1143,7 @@
     </row>
     <row r="6" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4">
         <v>180</v>
@@ -1130,7 +1151,7 @@
     </row>
     <row r="7" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D7" s="4">
         <v>80</v>
@@ -1138,7 +1159,7 @@
     </row>
     <row r="8" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D8" s="4">
         <v>140</v>
@@ -1146,7 +1167,7 @@
     </row>
     <row r="9" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D9" s="4">
         <v>130</v>
@@ -1154,7 +1175,7 @@
     </row>
     <row r="10" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="D10" s="4">
         <v>220</v>
@@ -1162,7 +1183,7 @@
     </row>
     <row r="11" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D11" s="4">
         <v>100</v>
@@ -1170,7 +1191,7 @@
     </row>
     <row r="12" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D12" s="4">
         <v>150</v>
@@ -1178,7 +1199,7 @@
     </row>
     <row r="13" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D13" s="4">
         <v>160</v>
@@ -1186,7 +1207,7 @@
     </row>
     <row r="14" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="D14" s="15">
         <v>1300</v>
@@ -1194,7 +1215,7 @@
     </row>
     <row r="15" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B15" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="13">
@@ -1204,7 +1225,7 @@
     </row>
     <row r="16" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B16" s="7" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D16" s="4">
         <v>120</v>
@@ -1212,7 +1233,7 @@
     </row>
     <row r="17" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B17" s="7" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D17" s="4">
         <v>150</v>
@@ -1220,7 +1241,7 @@
     </row>
     <row r="18" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D18" s="4">
         <v>270</v>
@@ -1228,7 +1249,7 @@
     </row>
     <row r="19" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B19" s="7" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D19" s="4">
         <v>300</v>
@@ -1236,7 +1257,7 @@
     </row>
     <row r="20" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B20" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D20" s="4">
         <v>150</v>
@@ -1244,7 +1265,7 @@
     </row>
     <row r="21" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D21" s="4">
         <v>360</v>
@@ -1252,7 +1273,7 @@
     </row>
     <row r="22" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="D22" s="4">
         <v>225</v>
@@ -1260,7 +1281,7 @@
     </row>
     <row r="23" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B23" s="7" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D23" s="4">
         <v>210</v>
@@ -1268,7 +1289,7 @@
     </row>
     <row r="24" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B24" s="7" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="D24" s="4">
         <v>240</v>
@@ -1276,7 +1297,7 @@
     </row>
     <row r="25" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B25" s="7" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="D25" s="4">
         <v>240</v>
@@ -1284,7 +1305,7 @@
     </row>
     <row r="26" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B26" s="7" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="D26" s="4">
         <v>450</v>
@@ -1292,7 +1313,7 @@
     </row>
     <row r="27" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D27" s="4">
         <v>360</v>
@@ -1300,7 +1321,7 @@
     </row>
     <row r="28" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="D28" s="4">
         <v>270</v>
@@ -1308,7 +1329,7 @@
     </row>
     <row r="29" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B29" s="7" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D29" s="4">
         <v>240</v>
@@ -1316,7 +1337,7 @@
     </row>
     <row r="30" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B30" s="7" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D30" s="4">
         <v>300</v>
@@ -1324,7 +1345,7 @@
     </row>
     <row r="31" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B31" s="7" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="D31" s="4">
         <v>240</v>
@@ -1332,7 +1353,7 @@
     </row>
     <row r="32" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B32" s="7" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="D32" s="4">
         <v>485</v>
@@ -1340,7 +1361,7 @@
     </row>
     <row r="33" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B33" s="7" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D33" s="4">
         <v>390</v>
@@ -1348,7 +1369,7 @@
     </row>
     <row r="34" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B34" s="7" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D34" s="4">
         <v>500</v>
@@ -1356,7 +1377,7 @@
     </row>
     <row r="35" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B35" s="7" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D35" s="4">
         <v>-500</v>
@@ -1364,7 +1385,7 @@
     </row>
     <row r="36" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B36" s="7" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="D36" s="4">
         <v>-400</v>
@@ -1372,7 +1393,7 @@
     </row>
     <row r="37" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B37" s="7" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D37" s="4">
         <v>-300</v>
@@ -1380,7 +1401,7 @@
     </row>
     <row r="38" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B38" s="7" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D38" s="4">
         <v>-650</v>
@@ -1388,7 +1409,7 @@
     </row>
     <row r="39" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B39" s="7" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="D39" s="4">
         <v>-650</v>
@@ -1396,7 +1417,7 @@
     </row>
     <row r="40" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B40" s="7" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="D40" s="4">
         <v>-650</v>
@@ -1404,7 +1425,7 @@
     </row>
     <row r="41" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B41" s="7" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="D41" s="4">
         <v>-400</v>
@@ -1412,7 +1433,7 @@
     </row>
     <row r="42" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B42" s="7" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="D42" s="4">
         <v>-2030</v>
@@ -1420,7 +1441,7 @@
     </row>
     <row r="43" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B43" s="7" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D43" s="4">
         <v>-600</v>
@@ -1428,7 +1449,7 @@
     </row>
     <row r="44" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B44" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C44" s="17"/>
       <c r="D44" s="13">
@@ -1438,14 +1459,14 @@
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B46" s="6" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="C46" s="11"/>
       <c r="D46" s="11"/>
     </row>
     <row r="47" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B47" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="D47" s="4">
         <v>300</v>
@@ -1453,7 +1474,7 @@
     </row>
     <row r="48" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B48" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C48" s="17"/>
       <c r="D48" s="13">
@@ -1463,14 +1484,14 @@
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B50" s="6" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="C50" s="11"/>
       <c r="D50" s="11"/>
     </row>
     <row r="51" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B51" s="3" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="D51" s="4">
         <v>650</v>
@@ -1478,7 +1499,7 @@
     </row>
     <row r="52" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B52" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C52" s="17"/>
       <c r="D52" s="13">
@@ -1488,7 +1509,7 @@
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B53" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C53" s="17"/>
       <c r="D53" s="13">
@@ -1498,14 +1519,14 @@
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B55" s="6" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="C55" s="11"/>
       <c r="D55" s="11"/>
     </row>
     <row r="56" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B56" s="3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D56" s="4">
         <v>50</v>
@@ -1513,7 +1534,7 @@
     </row>
     <row r="57" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B57" s="3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D57" s="4">
         <v>40</v>
@@ -1521,7 +1542,7 @@
     </row>
     <row r="58" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B58" s="3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="D58" s="4">
         <v>20</v>
@@ -1529,7 +1550,7 @@
     </row>
     <row r="59" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B59" s="3" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="D59" s="4">
         <v>40</v>
@@ -1537,7 +1558,7 @@
     </row>
     <row r="60" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B60" s="3" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="D60" s="4">
         <v>20</v>
@@ -1545,7 +1566,7 @@
     </row>
     <row r="61" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B61" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="D61" s="4">
         <v>20</v>
@@ -1553,7 +1574,7 @@
     </row>
     <row r="62" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B62" s="3" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D62" s="4">
         <v>10</v>
@@ -1561,7 +1582,7 @@
     </row>
     <row r="63" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B63" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C63" s="17"/>
       <c r="D63" s="13">
@@ -1571,7 +1592,7 @@
     </row>
     <row r="64" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B64" s="3" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="D64" s="4">
         <v>150</v>
@@ -1579,7 +1600,7 @@
     </row>
     <row r="65" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B65" s="3" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="D65" s="4">
         <v>160</v>
@@ -1587,7 +1608,7 @@
     </row>
     <row r="66" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B66" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="D66" s="4">
         <v>90</v>
@@ -1595,7 +1616,7 @@
     </row>
     <row r="67" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B67" s="3" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="D67" s="4">
         <v>60</v>
@@ -1603,7 +1624,7 @@
     </row>
     <row r="68" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B68" s="3" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="D68" s="4">
         <v>40</v>
@@ -1611,7 +1632,7 @@
     </row>
     <row r="69" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B69" s="3" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="D69" s="4">
         <v>120</v>
@@ -1619,7 +1640,7 @@
     </row>
     <row r="70" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B70" s="3" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="D70" s="4">
         <v>105</v>
@@ -1627,7 +1648,7 @@
     </row>
     <row r="71" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B71" s="3" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D71" s="4">
         <v>75</v>
@@ -1635,7 +1656,7 @@
     </row>
     <row r="72" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B72" s="3" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D72" s="4">
         <v>60</v>
@@ -1643,7 +1664,7 @@
     </row>
     <row r="73" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B73" s="3" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="D73" s="4">
         <v>40</v>
@@ -1651,7 +1672,7 @@
     </row>
     <row r="74" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B74" s="3" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="D74" s="4">
         <v>130</v>
@@ -1659,7 +1680,7 @@
     </row>
     <row r="75" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B75" s="3" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="D75" s="4">
         <v>70</v>
@@ -1667,7 +1688,7 @@
     </row>
     <row r="76" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B76" s="3" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="D76" s="4">
         <v>50</v>
@@ -1675,7 +1696,7 @@
     </row>
     <row r="77" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B77" s="3" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D77" s="4">
         <v>30</v>
@@ -1683,7 +1704,7 @@
     </row>
     <row r="78" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B78" s="3" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="D78" s="4">
         <v>20</v>
@@ -1691,7 +1712,7 @@
     </row>
     <row r="79" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B79" s="3" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="D79" s="4">
         <v>-10</v>
@@ -1699,7 +1720,7 @@
     </row>
     <row r="80" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B80" s="3" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="D80" s="4">
         <v>-25</v>
@@ -1707,7 +1728,7 @@
     </row>
     <row r="81" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B81" s="3" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="D81" s="4">
         <v>-95</v>
@@ -1715,7 +1736,7 @@
     </row>
     <row r="82" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B82" s="3" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="D82" s="4">
         <v>-60</v>
@@ -1723,7 +1744,7 @@
     </row>
     <row r="83" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B83" s="3" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D83" s="4">
         <v>-40</v>
@@ -1731,7 +1752,7 @@
     </row>
     <row r="84" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B84" s="3" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D84" s="4">
         <v>-65</v>
@@ -1739,7 +1760,7 @@
     </row>
     <row r="85" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B85" s="3" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="D85" s="4">
         <v>-35</v>
@@ -1747,7 +1768,7 @@
     </row>
     <row r="86" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B86" s="3" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="D86" s="4">
         <v>-25</v>
@@ -1755,7 +1776,7 @@
     </row>
     <row r="87" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B87" s="3" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="D87" s="4">
         <v>-125</v>
@@ -1763,7 +1784,7 @@
     </row>
     <row r="88" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B88" s="3" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="D88" s="4">
         <v>-55</v>
@@ -1771,7 +1792,7 @@
     </row>
     <row r="89" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B89" s="3" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="D89" s="4">
         <v>-45</v>
@@ -1779,7 +1800,7 @@
     </row>
     <row r="90" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B90" s="3" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="D90" s="4">
         <v>-100</v>
@@ -1787,7 +1808,7 @@
     </row>
     <row r="91" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B91" s="3" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="D91" s="4">
         <v>-80</v>
@@ -1795,7 +1816,7 @@
     </row>
     <row r="92" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B92" s="3" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="D92" s="4">
         <v>-25</v>
@@ -1803,7 +1824,7 @@
     </row>
     <row r="93" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B93" s="3" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="D93" s="4">
         <v>-129</v>
@@ -1811,7 +1832,7 @@
     </row>
     <row r="94" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B94" s="3" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="D94" s="4">
         <v>-70</v>
@@ -1819,7 +1840,7 @@
     </row>
     <row r="95" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B95" s="3" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="D95" s="4">
         <v>-105</v>
@@ -1827,7 +1848,7 @@
     </row>
     <row r="96" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B96" s="3" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="D96" s="4">
         <v>-75</v>
@@ -1835,7 +1856,7 @@
     </row>
     <row r="97" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B97" s="3" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="D97" s="4">
         <v>-36</v>
@@ -1843,7 +1864,7 @@
     </row>
     <row r="98" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B98" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C98" s="17"/>
       <c r="D98" s="13">
@@ -1853,14 +1874,14 @@
     </row>
     <row r="100" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B100" s="6" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="C100" s="11"/>
       <c r="D100" s="11"/>
     </row>
     <row r="101" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B101" s="3" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="D101" s="4">
         <v>200</v>
@@ -1868,7 +1889,7 @@
     </row>
     <row r="102" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B102" s="3" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="D102" s="4">
         <v>180</v>
@@ -1876,7 +1897,7 @@
     </row>
     <row r="103" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B103" s="3" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="D103" s="4">
         <v>130</v>
@@ -1884,7 +1905,7 @@
     </row>
     <row r="104" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B104" s="3" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="D104" s="4">
         <v>170</v>
@@ -1892,7 +1913,7 @@
     </row>
     <row r="105" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B105" s="3" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="D105" s="4">
         <v>65</v>
@@ -1900,7 +1921,7 @@
     </row>
     <row r="106" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B106" s="3" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D106" s="4">
         <v>95</v>
@@ -1908,7 +1929,7 @@
     </row>
     <row r="107" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B107" s="3" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="D107" s="4">
         <v>45</v>
@@ -1916,7 +1937,7 @@
     </row>
     <row r="108" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B108" s="3" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="D108" s="4">
         <v>40</v>
@@ -1924,7 +1945,7 @@
     </row>
     <row r="109" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B109" s="3" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="D109" s="4">
         <v>35</v>
@@ -1932,7 +1953,7 @@
     </row>
     <row r="110" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B110" s="3" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="D110" s="4">
         <v>20</v>
@@ -1940,7 +1961,7 @@
     </row>
     <row r="111" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B111" s="3" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="D111" s="4">
         <v>90</v>
@@ -1948,7 +1969,7 @@
     </row>
     <row r="112" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B112" s="3" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="D112" s="4">
         <v>70</v>
@@ -1956,7 +1977,7 @@
     </row>
     <row r="113" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B113" s="3" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="D113" s="4">
         <v>60</v>
@@ -1964,7 +1985,7 @@
     </row>
     <row r="114" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B114" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C114" s="17"/>
       <c r="D114" s="13">
@@ -1974,7 +1995,7 @@
     </row>
     <row r="115" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B115" s="3" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="D115" s="4">
         <v>400</v>
@@ -1982,7 +2003,7 @@
     </row>
     <row r="116" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B116" s="3" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="D116" s="4">
         <v>-160</v>
@@ -1990,7 +2011,7 @@
     </row>
     <row r="117" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B117" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C117" s="17"/>
       <c r="D117" s="13">
@@ -2000,14 +2021,14 @@
     </row>
     <row r="119" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B119" s="6" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="C119" s="11"/>
       <c r="D119" s="11"/>
     </row>
     <row r="120" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B120" s="3" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="D120" s="4">
         <v>250</v>
@@ -2015,7 +2036,7 @@
     </row>
     <row r="121" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B121" s="3" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="D121" s="4">
         <v>200</v>
@@ -2023,7 +2044,7 @@
     </row>
     <row r="122" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B122" s="3" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="D122" s="4">
         <v>180</v>
@@ -2031,7 +2052,7 @@
     </row>
     <row r="123" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B123" s="3" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="D123" s="4">
         <v>120</v>
@@ -2039,7 +2060,7 @@
     </row>
     <row r="124" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B124" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C124" s="17"/>
       <c r="D124" s="13">
@@ -2049,7 +2070,7 @@
     </row>
     <row r="125" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B125" s="3" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="D125" s="4">
         <v>-40</v>
@@ -2057,7 +2078,7 @@
     </row>
     <row r="126" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B126" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C126" s="17"/>
       <c r="D126" s="13">
@@ -2067,14 +2088,14 @@
     </row>
     <row r="128" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B128" s="6" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="C128" s="11"/>
       <c r="D128" s="11"/>
     </row>
     <row r="129" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B129" s="3" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="D129" s="4">
         <v>610</v>
@@ -2082,7 +2103,7 @@
     </row>
     <row r="130" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B130" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C130" s="17"/>
       <c r="D130" s="13">
@@ -2092,7 +2113,7 @@
     </row>
     <row r="131" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B131" s="3" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="D131" s="4">
         <v>-30</v>
@@ -2100,7 +2121,7 @@
     </row>
     <row r="132" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B132" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C132" s="17"/>
       <c r="D132" s="13">
@@ -2129,19 +2150,19 @@
   <sheetData>
     <row r="1" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B3" s="3" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="D3" s="4">
         <v>300</v>
@@ -2149,7 +2170,7 @@
     </row>
     <row r="4" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="D4" s="4">
         <v>180</v>
@@ -2157,7 +2178,7 @@
     </row>
     <row r="5" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="D5" s="4">
         <v>130</v>
@@ -2165,7 +2186,7 @@
     </row>
     <row r="6" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="D6" s="4">
         <v>170</v>
@@ -2173,7 +2194,7 @@
     </row>
     <row r="7" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="D7" s="4">
         <v>750</v>
@@ -2181,7 +2202,7 @@
     </row>
     <row r="8" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="D8" s="4">
         <v>500</v>
@@ -2189,7 +2210,7 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B9" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="13">
@@ -2199,7 +2220,7 @@
     </row>
     <row r="10" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="D10" s="4">
         <v>-2030</v>
@@ -2207,7 +2228,7 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="13">
@@ -2217,14 +2238,14 @@
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B13" s="6" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
     </row>
     <row r="14" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="D14" s="4">
         <v>220</v>
@@ -2232,7 +2253,7 @@
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B15" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="13">
@@ -2242,7 +2263,7 @@
     </row>
     <row r="16" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="D16" s="4">
         <v>-220</v>
@@ -2250,7 +2271,7 @@
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="13">
@@ -2279,19 +2300,19 @@
   <sheetData>
     <row r="1" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
-        <v>120</v>
+        <v>3</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
     </row>
     <row r="3" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B3" s="3" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="D3" s="4">
         <v>160</v>
@@ -2299,7 +2320,7 @@
     </row>
     <row r="4" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="D4" s="4">
         <v>610</v>
@@ -2307,7 +2328,7 @@
     </row>
     <row r="5" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="D5" s="4">
         <v>220</v>
@@ -2315,7 +2336,7 @@
     </row>
     <row r="6" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D6" s="4">
         <v>1300</v>
@@ -2323,7 +2344,7 @@
     </row>
     <row r="7" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B7" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="13">
@@ -2333,7 +2354,7 @@
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C8" s="17"/>
       <c r="D8" s="13">
@@ -2343,14 +2364,14 @@
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B10" s="6" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
     </row>
     <row r="11" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="D11" s="4">
         <v>340</v>
@@ -2358,7 +2379,7 @@
     </row>
     <row r="12" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="D12" s="4">
         <v>180</v>
@@ -2366,7 +2387,7 @@
     </row>
     <row r="13" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="D13" s="4">
         <v>80</v>
@@ -2374,7 +2395,7 @@
     </row>
     <row r="14" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="D14" s="4">
         <v>140</v>
@@ -2382,7 +2403,7 @@
     </row>
     <row r="15" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="D15" s="4">
         <v>130</v>
@@ -2390,7 +2411,7 @@
     </row>
     <row r="16" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B16" s="3" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="D16" s="4">
         <v>100</v>
@@ -2398,7 +2419,7 @@
     </row>
     <row r="17" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B17" s="3" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="D17" s="4">
         <v>150</v>
@@ -2406,7 +2427,7 @@
     </row>
     <row r="18" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B18" s="3" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="D18" s="4">
         <v>-300</v>
@@ -2414,7 +2435,7 @@
     </row>
     <row r="19" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B19" s="3" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="D19" s="4">
         <v>-650</v>
@@ -2422,7 +2443,7 @@
     </row>
     <row r="20" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B20" s="16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="13">
@@ -2432,7 +2453,7 @@
     </row>
     <row r="21" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B21" s="3" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="D21" s="4">
         <v>-650</v>
@@ -2440,7 +2461,7 @@
     </row>
     <row r="22" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B22" s="3" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="D22" s="4">
         <v>120</v>
@@ -2448,7 +2469,7 @@
     </row>
     <row r="23" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B23" s="3" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="D23" s="4">
         <v>-10</v>
@@ -2456,7 +2477,7 @@
     </row>
     <row r="24" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B24" s="3" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D24" s="4">
         <v>150</v>
@@ -2464,7 +2485,7 @@
     </row>
     <row r="25" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B25" s="3" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D25" s="4">
         <v>270</v>
@@ -2472,7 +2493,7 @@
     </row>
     <row r="26" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B26" s="3" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="D26" s="4">
         <v>-25</v>
@@ -2480,7 +2501,7 @@
     </row>
     <row r="27" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B27" s="3" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D27" s="4">
         <v>300</v>
@@ -2488,7 +2509,7 @@
     </row>
     <row r="28" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B28" s="3" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="D28" s="4">
         <v>-95</v>
@@ -2496,7 +2517,7 @@
     </row>
     <row r="29" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B29" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D29" s="4">
         <v>150</v>
@@ -2504,7 +2525,7 @@
     </row>
     <row r="30" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B30" s="3" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="D30" s="4">
         <v>360</v>
@@ -2512,7 +2533,7 @@
     </row>
     <row r="31" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B31" s="3" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="D31" s="4">
         <v>-60</v>
@@ -2520,7 +2541,7 @@
     </row>
     <row r="32" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B32" s="3" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="D32" s="4">
         <v>225</v>
@@ -2528,7 +2549,7 @@
     </row>
     <row r="33" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B33" s="3" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D33" s="4">
         <v>-40</v>
@@ -2536,7 +2557,7 @@
     </row>
     <row r="34" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B34" s="3" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="D34" s="4">
         <v>210</v>
@@ -2544,7 +2565,7 @@
     </row>
     <row r="35" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B35" s="3" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D35" s="4">
         <v>-65</v>
@@ -2552,7 +2573,7 @@
     </row>
     <row r="36" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B36" s="3" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="D36" s="4">
         <v>-650</v>
@@ -2560,7 +2581,7 @@
     </row>
     <row r="37" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B37" s="3" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="D37" s="4">
         <v>240</v>
@@ -2568,7 +2589,7 @@
     </row>
     <row r="38" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B38" s="3" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="D38" s="4">
         <v>-35</v>
@@ -2576,7 +2597,7 @@
     </row>
     <row r="39" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B39" s="3" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="D39" s="4">
         <v>240</v>
@@ -2584,7 +2605,7 @@
     </row>
     <row r="40" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B40" s="3" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="D40" s="4">
         <v>-25</v>
@@ -2592,7 +2613,7 @@
     </row>
     <row r="41" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B41" s="3" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="D41" s="4">
         <v>450</v>
@@ -2600,7 +2621,7 @@
     </row>
     <row r="42" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B42" s="3" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="D42" s="4">
         <v>-125</v>
@@ -2608,7 +2629,7 @@
     </row>
     <row r="43" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B43" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D43" s="4">
         <v>360</v>
@@ -2616,7 +2637,7 @@
     </row>
     <row r="44" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B44" s="3" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="D44" s="4">
         <v>-55</v>
@@ -2624,7 +2645,7 @@
     </row>
     <row r="45" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B45" s="3" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="D45" s="4">
         <v>270</v>
@@ -2632,7 +2653,7 @@
     </row>
     <row r="46" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B46" s="3" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="D46" s="4">
         <v>-45</v>
@@ -2640,7 +2661,7 @@
     </row>
     <row r="47" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B47" s="3" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D47" s="4">
         <v>240</v>
@@ -2648,7 +2669,7 @@
     </row>
     <row r="48" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B48" s="3" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="D48" s="4">
         <v>-100</v>
@@ -2656,7 +2677,7 @@
     </row>
     <row r="49" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B49" s="3" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D49" s="4">
         <v>300</v>
@@ -2664,7 +2685,7 @@
     </row>
     <row r="50" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B50" s="3" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="D50" s="4">
         <v>-80</v>
@@ -2672,7 +2693,7 @@
     </row>
     <row r="51" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B51" s="3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="D51" s="4">
         <v>-650</v>
@@ -2680,7 +2701,7 @@
     </row>
     <row r="52" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B52" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="D52" s="4">
         <v>240</v>
@@ -2688,7 +2709,7 @@
     </row>
     <row r="53" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B53" s="3" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="D53" s="4">
         <v>-25</v>
@@ -2696,7 +2717,7 @@
     </row>
     <row r="54" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B54" s="3" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="D54" s="4">
         <v>485</v>
@@ -2704,7 +2725,7 @@
     </row>
     <row r="55" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B55" s="3" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="D55" s="4">
         <v>-129</v>
@@ -2712,7 +2733,7 @@
     </row>
     <row r="56" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B56" s="3" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D56" s="4">
         <v>390</v>
@@ -2720,7 +2741,7 @@
     </row>
     <row r="57" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B57" s="3" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="D57" s="4">
         <v>-70</v>
@@ -2728,7 +2749,7 @@
     </row>
     <row r="58" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B58" s="3" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D58" s="4">
         <v>500</v>
@@ -2736,7 +2757,7 @@
     </row>
     <row r="59" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B59" s="3" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="D59" s="4">
         <v>-105</v>
@@ -2744,7 +2765,7 @@
     </row>
     <row r="60" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B60" s="3" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="D60" s="4">
         <v>300</v>
@@ -2752,7 +2773,7 @@
     </row>
     <row r="61" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B61" s="3" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="D61" s="4">
         <v>-75</v>
@@ -2760,7 +2781,7 @@
     </row>
     <row r="62" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B62" s="3" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="D62" s="4">
         <v>220</v>
@@ -2768,7 +2789,7 @@
     </row>
     <row r="63" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B63" s="3" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="D63" s="4">
         <v>-36</v>
@@ -2776,7 +2797,7 @@
     </row>
     <row r="64" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B64" s="3" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D64" s="4">
         <v>-160</v>
@@ -2784,7 +2805,7 @@
     </row>
     <row r="65" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B65" s="3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="D65" s="4">
         <v>-40</v>
@@ -2792,7 +2813,7 @@
     </row>
     <row r="66" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B66" s="3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="D66" s="4">
         <v>-30</v>
@@ -2800,7 +2821,7 @@
     </row>
     <row r="67" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B67" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C67" s="17"/>
       <c r="D67" s="13">
@@ -2810,14 +2831,14 @@
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B69" s="6" t="s">
-        <v>143</v>
+        <v>8</v>
       </c>
       <c r="C69" s="11"/>
       <c r="D69" s="11"/>
     </row>
     <row r="70" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B70" s="3" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="D70" s="4">
         <v>-600</v>
@@ -2825,7 +2846,7 @@
     </row>
     <row r="71" spans="2:4" collapsed="1" x14ac:dyDescent="0.2">
       <c r="B71" s="16" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C71" s="17"/>
       <c r="D71" s="13">
@@ -2861,235 +2882,207 @@
   <sheetData>
     <row r="1" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="2"/>
       <c r="C3" s="12" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B4" s="9" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" s="8" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C5" s="19">
-        <f>Assets!D15</f>
         <v>1300</v>
       </c>
       <c r="D5" s="19">
-        <f>Assets!D44</f>
         <v>620</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" s="8" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="C6" s="20">
         <v>0</v>
       </c>
       <c r="D6" s="20">
-        <f>Assets!D48</f>
         <v>300</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" s="8" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="C7" s="20">
-        <f>Assets!D52</f>
         <v>650</v>
       </c>
       <c r="D7" s="20">
-        <f>Assets!D53</f>
         <v>650</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" s="8" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="C8" s="20">
-        <f>Assets!D63</f>
         <v>200</v>
       </c>
       <c r="D8" s="20">
-        <f>Assets!D98</f>
         <v>200</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B9" s="8" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="C9" s="20">
-        <f>Assets!D114</f>
         <v>1200</v>
       </c>
       <c r="D9" s="20">
-        <f>Assets!D117</f>
         <v>1440</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B10" s="8" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="C10" s="20">
-        <f>Assets!D124</f>
         <v>750</v>
       </c>
       <c r="D10" s="20">
-        <f>Assets!D126</f>
         <v>710</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" s="8" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="C11" s="20">
-        <f>Assets!D130</f>
         <v>610</v>
       </c>
       <c r="D11" s="20">
-        <f>Assets!D132</f>
         <v>580</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="C12" s="21">
-        <f>SUM(C5:C11)</f>
         <v>4710</v>
       </c>
       <c r="D12" s="21">
-        <f>SUM(D5:D11)</f>
         <v>4500</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B13" s="9" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B14" s="8" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="C14" s="19">
-        <f>Liabilities!D9</f>
         <v>2030</v>
       </c>
       <c r="D14" s="19">
-        <f>Liabilities!D11</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B15" s="8" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="C15" s="20">
-        <f>Liabilities!D15</f>
         <v>220</v>
       </c>
       <c r="D15" s="20">
-        <f>Liabilities!D17</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B16" s="10" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C16" s="21">
-        <f>SUM(C14:C15)</f>
         <v>2250</v>
       </c>
       <c r="D16" s="21">
-        <f>SUM(D14:D15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="9" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B18" s="8" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C18" s="19">
-        <f>Reasons!D7</f>
         <v>2290</v>
       </c>
       <c r="D18" s="19">
-        <f>Reasons!D8</f>
         <v>2290</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B19" s="8" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="C19" s="20">
-        <f>Reasons!D20</f>
         <v>170</v>
       </c>
       <c r="D19" s="20">
-        <f>Reasons!D66</f>
-        <v>-30</v>
+        <v>2810</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" s="8" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C20" s="20">
         <v>0</v>
       </c>
       <c r="D20" s="20">
-        <f>Reasons!D70</f>
         <v>-600</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B21" s="10" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="C21" s="21">
-        <f>SUM(C18:C20)</f>
         <v>2460</v>
       </c>
       <c r="D21" s="21">
-        <f>SUM(D18:D20)</f>
-        <v>1660</v>
+        <v>4500</v>
       </c>
     </row>
   </sheetData>
@@ -3112,18 +3105,18 @@
   <sheetData>
     <row r="1" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="D2" s="4"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="22" t="s">
-        <v>157</v>
+        <v>2</v>
       </c>
       <c r="D3" s="4"/>
     </row>
@@ -3133,14 +3126,14 @@
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" s="29" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C5" s="29"/>
       <c r="D5" s="29"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" s="23" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="D6" s="30">
         <v>6020</v>
@@ -3148,7 +3141,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" s="25" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="27">
@@ -3158,14 +3151,14 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B9" s="29" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C9" s="29"/>
       <c r="D9" s="29"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B10" s="23" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="D10" s="30">
         <v>1200</v>
@@ -3173,7 +3166,7 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" s="23" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="D11" s="28">
         <v>1950</v>
@@ -3181,7 +3174,7 @@
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" s="23" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D12" s="28">
         <v>230</v>
@@ -3189,7 +3182,7 @@
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B13" s="25" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C13" s="26"/>
       <c r="D13" s="27">
@@ -3199,7 +3192,7 @@
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B15" s="25" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C15" s="26"/>
       <c r="D15" s="27">
@@ -3341,7 +3334,7 @@
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="B1:D17"/>
+  <dimension ref="B1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.33203125" customWidth="1"/>
@@ -3351,29 +3344,29 @@
   <sheetData>
     <row r="1" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>167</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="22" t="s">
-        <v>157</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" s="29" t="s">
-        <v>120</v>
+        <v>3</v>
       </c>
       <c r="C5" s="29"/>
       <c r="D5" s="29"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" s="23" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D6" s="24">
         <v>2290</v>
@@ -3381,7 +3374,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" s="25" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C7" s="26"/>
       <c r="D7" s="27">
@@ -3394,14 +3387,14 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B9" s="29" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="C9" s="29"/>
       <c r="D9" s="29"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B10" s="23" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D10" s="24">
         <v>170</v>
@@ -3409,7 +3402,7 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" s="23" t="s">
-        <v>168</v>
+        <v>7</v>
       </c>
       <c r="D11" s="28">
         <v>2640</v>
@@ -3417,7 +3410,7 @@
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" s="25" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C12" s="26"/>
       <c r="D12" s="27">
@@ -3430,14 +3423,14 @@
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B14" s="29" t="s">
-        <v>143</v>
+        <v>8</v>
       </c>
       <c r="C14" s="29"/>
       <c r="D14" s="29"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B15" s="23" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D15" s="24">
         <v>0</v>
@@ -3445,7 +3438,7 @@
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B16" s="23" t="s">
-        <v>169</v>
+        <v>9</v>
       </c>
       <c r="D16" s="28">
         <v>-600</v>
@@ -3453,7 +3446,7 @@
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="25" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C17" s="26"/>
       <c r="D17" s="27">
@@ -3461,6 +3454,31 @@
         <v>-600</v>
       </c>
     </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="19">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="20">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="32">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" ht="16" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3481,30 +3499,30 @@
   <sheetData>
     <row r="1" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>145</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:4" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D2" s="4"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="22" t="s">
-        <v>157</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" s="29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C5" s="29"/>
       <c r="D5" s="29"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" s="23" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D6" s="30">
         <v>5500</v>
@@ -3512,7 +3530,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" s="23" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D7" s="28">
         <v>-1200</v>
@@ -3520,7 +3538,7 @@
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" s="23" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D8" s="28">
         <v>-1950</v>
@@ -3528,7 +3546,7 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B9" s="25" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C9" s="26"/>
       <c r="D9" s="27">
@@ -3538,14 +3556,14 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" s="29" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C11" s="29"/>
       <c r="D11" s="29"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" s="23" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D12" s="30">
         <v>-400</v>
@@ -3553,7 +3571,7 @@
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B13" s="25" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C13" s="26"/>
       <c r="D13" s="27">
@@ -3563,14 +3581,14 @@
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B15" s="29" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C15" s="29"/>
       <c r="D15" s="29"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B16" s="23" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D16" s="30">
         <v>-2030</v>
@@ -3578,7 +3596,7 @@
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="23" t="s">
-        <v>169</v>
+        <v>9</v>
       </c>
       <c r="D17" s="28">
         <v>-600</v>
@@ -3586,7 +3604,7 @@
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B18" s="25" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C18" s="26"/>
       <c r="D18" s="27">
@@ -3596,7 +3614,7 @@
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" s="25" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C20" s="26"/>
       <c r="D20" s="27">
@@ -3606,7 +3624,7 @@
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B21" s="23" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D21" s="31">
         <v>1300</v>
@@ -3614,7 +3632,7 @@
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B22" s="25" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C22" s="26"/>
       <c r="D22" s="27">

</xml_diff>

<commit_message>
Workbooks: restore Accounts Receivable section visibility
The generic ledger rebuild swept AR's header row into a hidden outline
group (AR wasn't in the account list), so 32-2 page 2 showed no AR under
Assets. Restored the original design in all seven post-receivable
workbooks: header level-0 visible, Ridgeline row grouped but shipped
expanded, balance not collapsed. Recached, regenerated, 20/20
invariants; 32-2 pages browser-verified side by side.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bike-Repair-Source-Workbooks/Bike-Repair-End.xlsx
+++ b/Bike-Repair-Source-Workbooks/Bike-Repair-End.xlsx
@@ -917,7 +917,7 @@
       <c r="B34" s="7" t="n"/>
       <c r="D34" s="4" t="n"/>
     </row>
-    <row r="35" hidden="1" outlineLevel="1">
+    <row r="35">
       <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Accounts Receivable</t>
@@ -926,7 +926,7 @@
       <c r="C35" s="11" t="n"/>
       <c r="D35" s="11" t="n"/>
     </row>
-    <row r="36" hidden="1" outlineLevel="1">
+    <row r="36" outlineLevel="1">
       <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Ridgeline Trail Crew — finished Aug 28, net 15 (unpaid)</t>
@@ -936,7 +936,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="37" collapsed="1">
+    <row r="37">
       <c r="B37" s="16" t="inlineStr">
         <is>
           <t>Balance, August 31, 2026</t>

</xml_diff>